<commit_message>
Read the Die temperature and sum volts with the command RDSTAT.
</commit_message>
<xml_diff>
--- a/src/drivers/adbms/ltc6812_on_core2/docs/Complete_BorgWarner_Gen3_0_CAN_Communication_Matrix.xlsx
+++ b/src/drivers/adbms/ltc6812_on_core2/docs/Complete_BorgWarner_Gen3_0_CAN_Communication_Matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\Aurix\Ecu8Tr\ADI\adbms6830_ws\ecu8tr_freertos_illd_adbms6830\src\drivers\adbms\ltc6812_on_core2\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2762098F-4F6D-47A8-B2FE-7C38EB446EDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88DFFCA0-59CE-4330-9451-5D5C98BD82A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31500" yWindow="17388" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Messages" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="370">
   <si>
     <t>Message Name</t>
   </si>
@@ -1122,6 +1122,15 @@
   </si>
   <si>
     <t>Done in code</t>
+  </si>
+  <si>
+    <t>Done in code, Transmiting rate: 1 time/s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done in code </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done in code, but instead of the cell, I used the terminal max and min </t>
   </si>
 </sst>
 </file>
@@ -1216,7 +1225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1227,7 +1236,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1237,6 +1246,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1708,6 +1720,9 @@
       <c r="C14" s="6" t="s">
         <v>41</v>
       </c>
+      <c r="D14" s="7" t="s">
+        <v>366</v>
+      </c>
     </row>
     <row r="15" spans="1:4" s="7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
@@ -1719,6 +1734,9 @@
       <c r="C15" s="6" t="s">
         <v>44</v>
       </c>
+      <c r="D15" s="7" t="s">
+        <v>366</v>
+      </c>
     </row>
     <row r="16" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
@@ -1730,8 +1748,9 @@
       <c r="C16" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="246.5" x14ac:dyDescent="0.35">
+      <c r="D16" s="7"/>
+    </row>
+    <row r="17" spans="1:4" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>48</v>
       </c>
@@ -1742,7 +1761,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>51</v>
       </c>
@@ -1752,8 +1771,9 @@
       <c r="C18" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D18" s="7"/>
+    </row>
+    <row r="19" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>54</v>
       </c>
@@ -1763,8 +1783,9 @@
       <c r="C19" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D19" s="7"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>57</v>
       </c>
@@ -1774,8 +1795,9 @@
       <c r="C20" s="2" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" ht="87" x14ac:dyDescent="0.35">
+      <c r="D20" s="7"/>
+    </row>
+    <row r="21" spans="1:4" ht="87" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>60</v>
       </c>
@@ -1786,18 +1808,21 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:4" s="7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A22" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="6" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" ht="261" x14ac:dyDescent="0.35">
+      <c r="D22" s="9" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="261" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>66</v>
       </c>
@@ -1808,7 +1833,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>69</v>
       </c>
@@ -1818,8 +1843,9 @@
       <c r="C24" s="2" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D24" s="7"/>
+    </row>
+    <row r="25" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>72</v>
       </c>
@@ -1829,8 +1855,9 @@
       <c r="C25" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D25" s="7"/>
+    </row>
+    <row r="26" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>75</v>
       </c>
@@ -1840,8 +1867,9 @@
       <c r="C26" s="2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D26" s="7"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>78</v>
       </c>
@@ -1851,8 +1879,9 @@
       <c r="C27" s="2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D27" s="7"/>
+    </row>
+    <row r="28" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>81</v>
       </c>
@@ -1862,8 +1891,9 @@
       <c r="C28" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D28" s="7"/>
+    </row>
+    <row r="29" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>84</v>
       </c>
@@ -1873,8 +1903,9 @@
       <c r="C29" s="2" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D29" s="7"/>
+    </row>
+    <row r="30" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>87</v>
       </c>
@@ -1884,8 +1915,9 @@
       <c r="C30" s="2" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D30" s="7"/>
+    </row>
+    <row r="31" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>90</v>
       </c>
@@ -1895,8 +1927,9 @@
       <c r="C31" s="2" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D31" s="7"/>
+    </row>
+    <row r="32" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="6" t="s">
         <v>93</v>
       </c>
@@ -1906,8 +1939,11 @@
       <c r="C32" s="6" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D32" s="7" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
         <v>96</v>
       </c>
@@ -1917,8 +1953,11 @@
       <c r="C33" s="6" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D33" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="6" t="s">
         <v>99</v>
       </c>
@@ -1928,8 +1967,11 @@
       <c r="C34" s="6" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D34" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" s="6" t="s">
         <v>102</v>
       </c>
@@ -1939,8 +1981,11 @@
       <c r="C35" s="6" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D35" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="6" t="s">
         <v>105</v>
       </c>
@@ -1950,8 +1995,11 @@
       <c r="C36" s="6" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D36" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="s">
         <v>108</v>
       </c>
@@ -1961,8 +2009,11 @@
       <c r="C37" s="6" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D37" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="6" t="s">
         <v>111</v>
       </c>
@@ -1972,8 +2023,11 @@
       <c r="C38" s="6" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D38" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="6" t="s">
         <v>114</v>
       </c>
@@ -1983,8 +2037,11 @@
       <c r="C39" s="6" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D39" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="6" t="s">
         <v>117</v>
       </c>
@@ -1994,8 +2051,11 @@
       <c r="C40" s="6" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D40" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="6" t="s">
         <v>120</v>
       </c>
@@ -2005,8 +2065,11 @@
       <c r="C41" s="6" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D41" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="6" t="s">
         <v>123</v>
       </c>
@@ -2016,8 +2079,11 @@
       <c r="C42" s="6" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D42" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
         <v>126</v>
       </c>
@@ -2027,8 +2093,11 @@
       <c r="C43" s="6" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D43" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="6" t="s">
         <v>129</v>
       </c>
@@ -2038,8 +2107,11 @@
       <c r="C44" s="6" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D44" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A45" s="6" t="s">
         <v>132</v>
       </c>
@@ -2049,8 +2121,11 @@
       <c r="C45" s="6" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D45" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="6" t="s">
         <v>135</v>
       </c>
@@ -2060,8 +2135,11 @@
       <c r="C46" s="6" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D46" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A47" s="6" t="s">
         <v>138</v>
       </c>
@@ -2071,8 +2149,11 @@
       <c r="C47" s="6" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D47" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="6" t="s">
         <v>141</v>
       </c>
@@ -2082,8 +2163,11 @@
       <c r="C48" s="6" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D48" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" s="6" t="s">
         <v>144</v>
       </c>
@@ -2093,8 +2177,11 @@
       <c r="C49" s="6" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D49" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A50" s="6" t="s">
         <v>147</v>
       </c>
@@ -2104,8 +2191,11 @@
       <c r="C50" s="6" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D50" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A51" s="6" t="s">
         <v>150</v>
       </c>
@@ -2115,8 +2205,11 @@
       <c r="C51" s="6" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" ht="217.5" x14ac:dyDescent="0.35">
+      <c r="D51" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>153</v>
       </c>
@@ -2127,7 +2220,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="53" spans="1:3" s="7" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" s="7" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A53" s="6" t="s">
         <v>156</v>
       </c>
@@ -2137,8 +2230,11 @@
       <c r="C53" s="6" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D53" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>159</v>
       </c>
@@ -2148,8 +2244,11 @@
       <c r="C54" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D54" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>161</v>
       </c>
@@ -2159,8 +2258,9 @@
       <c r="C55" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D55" s="7"/>
+    </row>
+    <row r="56" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>164</v>
       </c>
@@ -2170,8 +2270,9 @@
       <c r="C56" s="2" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D56" s="7"/>
+    </row>
+    <row r="57" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>167</v>
       </c>
@@ -2181,8 +2282,9 @@
       <c r="C57" s="2" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D57" s="7"/>
+    </row>
+    <row r="58" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>170</v>
       </c>
@@ -2192,19 +2294,23 @@
       <c r="C58" s="2" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A59" s="2" t="s">
+      <c r="D58" s="7"/>
+    </row>
+    <row r="59" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A59" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="B59" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="C59" s="2" t="s">
+      <c r="C59" s="6" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D59" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>176</v>
       </c>
@@ -2214,19 +2320,25 @@
       <c r="C60" s="2" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A61" s="2" t="s">
+      <c r="D60" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A61" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="B61" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="C61" s="2" t="s">
+      <c r="C61" s="6" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D61" s="7" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>182</v>
       </c>
@@ -2236,8 +2348,11 @@
       <c r="C62" s="2" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" ht="246.5" x14ac:dyDescent="0.35">
+      <c r="D62" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>185</v>
       </c>
@@ -2248,15 +2363,18 @@
         <v>187</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A64" s="2" t="s">
+    <row r="64" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A64" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="B64" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="C64" s="2" t="s">
+      <c r="C64" s="6" t="s">
         <v>190</v>
+      </c>
+      <c r="D64" s="7" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="203" x14ac:dyDescent="0.35">
@@ -2280,6 +2398,7 @@
       <c r="C66" s="2" t="s">
         <v>35</v>
       </c>
+      <c r="D66" s="7"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
@@ -2291,6 +2410,7 @@
       <c r="C67" s="2" t="s">
         <v>35</v>
       </c>
+      <c r="D67" s="7"/>
     </row>
     <row r="68" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A68" s="6" t="s">
@@ -2306,15 +2426,18 @@
         <v>366</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A69" s="2" t="s">
+    <row r="69" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="B69" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="C69" s="2" t="s">
+      <c r="C69" s="6" t="s">
         <v>203</v>
+      </c>
+      <c r="D69" s="7" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="203" x14ac:dyDescent="0.35">
@@ -2338,6 +2461,7 @@
       <c r="C71" s="2" t="s">
         <v>209</v>
       </c>
+      <c r="D71" s="7"/>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
@@ -2349,6 +2473,7 @@
       <c r="C72" s="2" t="s">
         <v>35</v>
       </c>
+      <c r="D72" s="7"/>
     </row>
     <row r="73" spans="1:4" ht="232" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
@@ -2371,6 +2496,7 @@
       <c r="C74" s="2" t="s">
         <v>217</v>
       </c>
+      <c r="D74" s="7"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
@@ -2382,6 +2508,7 @@
       <c r="C75" s="2" t="s">
         <v>220</v>
       </c>
+      <c r="D75" s="7"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
@@ -2393,6 +2520,7 @@
       <c r="C76" s="2" t="s">
         <v>223</v>
       </c>
+      <c r="D76" s="7"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
@@ -2404,6 +2532,7 @@
       <c r="C77" s="2" t="s">
         <v>226</v>
       </c>
+      <c r="D77" s="7"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
@@ -2415,6 +2544,7 @@
       <c r="C78" s="2" t="s">
         <v>229</v>
       </c>
+      <c r="D78" s="7"/>
     </row>
     <row r="79" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
@@ -2426,6 +2556,7 @@
       <c r="C79" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="D79" s="7"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
@@ -2437,8 +2568,9 @@
       <c r="C80" s="2" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D80" s="7"/>
+    </row>
+    <row r="81" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>236</v>
       </c>
@@ -2448,8 +2580,9 @@
       <c r="C81" s="2" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D81" s="7"/>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>239</v>
       </c>
@@ -2459,8 +2592,9 @@
       <c r="C82" s="2" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D82" s="7"/>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>242</v>
       </c>
@@ -2470,8 +2604,9 @@
       <c r="C83" s="2" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D83" s="7"/>
+    </row>
+    <row r="84" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>245</v>
       </c>
@@ -2481,8 +2616,9 @@
       <c r="C84" s="2" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D84" s="7"/>
+    </row>
+    <row r="85" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
         <v>248</v>
       </c>
@@ -2492,8 +2628,9 @@
       <c r="C85" s="2" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D85" s="7"/>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
         <v>251</v>
       </c>
@@ -2503,8 +2640,9 @@
       <c r="C86" s="2" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D86" s="7"/>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>254</v>
       </c>
@@ -2514,8 +2652,9 @@
       <c r="C87" s="2" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D87" s="7"/>
+    </row>
+    <row r="88" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>257</v>
       </c>
@@ -2525,8 +2664,9 @@
       <c r="C88" s="2" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D88" s="7"/>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>260</v>
       </c>
@@ -2536,8 +2676,9 @@
       <c r="C89" s="2" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D89" s="7"/>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
         <v>263</v>
       </c>
@@ -2547,8 +2688,9 @@
       <c r="C90" s="2" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="91" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D90" s="7"/>
+    </row>
+    <row r="91" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>266</v>
       </c>
@@ -2558,8 +2700,9 @@
       <c r="C91" s="2" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D91" s="7"/>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>269</v>
       </c>
@@ -2569,8 +2712,9 @@
       <c r="C92" s="2" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="93" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D92" s="7"/>
+    </row>
+    <row r="93" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>272</v>
       </c>
@@ -2580,8 +2724,9 @@
       <c r="C93" s="2" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="94" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D93" s="7"/>
+    </row>
+    <row r="94" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>275</v>
       </c>
@@ -2591,8 +2736,9 @@
       <c r="C94" s="2" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="95" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="D94" s="7"/>
+    </row>
+    <row r="95" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
         <v>278</v>
       </c>
@@ -2602,8 +2748,9 @@
       <c r="C95" s="2" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D95" s="7"/>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
         <v>281</v>
       </c>
@@ -2613,8 +2760,9 @@
       <c r="C96" s="2" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D96" s="7"/>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
         <v>284</v>
       </c>
@@ -2624,8 +2772,9 @@
       <c r="C97" s="2" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="98" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D97" s="7"/>
+    </row>
+    <row r="98" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
         <v>287</v>
       </c>
@@ -2635,8 +2784,9 @@
       <c r="C98" s="2" t="s">
         <v>289</v>
       </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D98" s="7"/>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
         <v>290</v>
       </c>
@@ -2646,8 +2796,9 @@
       <c r="C99" s="2" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D99" s="7"/>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>293</v>
       </c>
@@ -2657,8 +2808,9 @@
       <c r="C100" s="2" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D100" s="7"/>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
         <v>296</v>
       </c>
@@ -2668,8 +2820,9 @@
       <c r="C101" s="2" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D101" s="7"/>
+    </row>
+    <row r="102" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>299</v>
       </c>
@@ -2679,8 +2832,9 @@
       <c r="C102" s="2" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="103" spans="1:3" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="D102" s="7"/>
+    </row>
+    <row r="103" spans="1:4" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>302</v>
       </c>
@@ -2691,7 +2845,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>305</v>
       </c>
@@ -2701,8 +2855,9 @@
       <c r="C104" s="2" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D104" s="7"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>308</v>
       </c>
@@ -2712,8 +2867,9 @@
       <c r="C105" s="2" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D105" s="7"/>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>311</v>
       </c>
@@ -2723,8 +2879,9 @@
       <c r="C106" s="2" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="107" spans="1:3" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="D106" s="7"/>
+    </row>
+    <row r="107" spans="1:4" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>314</v>
       </c>
@@ -2735,7 +2892,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>317</v>
       </c>
@@ -2745,8 +2902,9 @@
       <c r="C108" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D108" s="7"/>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
         <v>319</v>
       </c>
@@ -2756,8 +2914,9 @@
       <c r="C109" s="2" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="110" spans="1:3" ht="232" x14ac:dyDescent="0.35">
+      <c r="D109" s="7"/>
+    </row>
+    <row r="110" spans="1:4" ht="232" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
         <v>322</v>
       </c>
@@ -2768,27 +2927,29 @@
         <v>324</v>
       </c>
     </row>
-    <row r="111" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A111" s="2" t="s">
+    <row r="111" spans="1:4" s="5" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A111" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="B111" s="2" t="s">
+      <c r="B111" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="C111" s="2" t="s">
+      <c r="C111" s="3" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A112" s="2" t="s">
+      <c r="D111" s="7"/>
+    </row>
+    <row r="112" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A112" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="B112" s="2" t="s">
+      <c r="B112" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="C112" s="2" t="s">
+      <c r="C112" s="3" t="s">
         <v>330</v>
       </c>
+      <c r="D112" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2800,7 +2961,7 @@
   <dimension ref="A1:A37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="53" customWidth="1"/>
+    <col min="1" max="1" width="65.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Instruct the .gitignore to ignore some files.
</commit_message>
<xml_diff>
--- a/src/drivers/adbms/ltc6812_on_core2/docs/Complete_BorgWarner_Gen3_0_CAN_Communication_Matrix.xlsx
+++ b/src/drivers/adbms/ltc6812_on_core2/docs/Complete_BorgWarner_Gen3_0_CAN_Communication_Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\Aurix\Ecu8Tr\ADI\adbms6830_ws\ecu8tr_freertos_illd_adbms6830\src\drivers\adbms\ltc6812_on_core2\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88DFFCA0-59CE-4330-9451-5D5C98BD82A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2605DFF-C91C-4D6D-ACA1-98AAB77B07C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="371">
   <si>
     <t>Message Name</t>
   </si>
@@ -1131,6 +1131,9 @@
   </si>
   <si>
     <t xml:space="preserve">Done in code, but instead of the cell, I used the terminal max and min </t>
+  </si>
+  <si>
+    <t>Done in code, set threashold UV OV UT OT</t>
   </si>
 </sst>
 </file>
@@ -1150,6 +1153,7 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1247,7 +1251,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2377,15 +2381,18 @@
         <v>366</v>
       </c>
     </row>
-    <row r="65" spans="1:4" ht="203" x14ac:dyDescent="0.35">
-      <c r="A65" s="2" t="s">
+    <row r="65" spans="1:4" s="7" customFormat="1" ht="203" x14ac:dyDescent="0.35">
+      <c r="A65" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="C65" s="2" t="s">
+      <c r="C65" s="6" t="s">
         <v>193</v>
+      </c>
+      <c r="D65" s="7" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
@@ -2440,15 +2447,18 @@
         <v>366</v>
       </c>
     </row>
-    <row r="70" spans="1:4" ht="203" x14ac:dyDescent="0.35">
-      <c r="A70" s="2" t="s">
+    <row r="70" spans="1:4" s="7" customFormat="1" ht="203" x14ac:dyDescent="0.35">
+      <c r="A70" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="C70" s="2" t="s">
+      <c r="C70" s="6" t="s">
         <v>206</v>
+      </c>
+      <c r="D70" s="7" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
@@ -2666,17 +2676,19 @@
       </c>
       <c r="D88" s="7"/>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A89" s="2" t="s">
+    <row r="89" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A89" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="B89" s="2" t="s">
+      <c r="B89" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="C89" s="2" t="s">
+      <c r="C89" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="D89" s="7"/>
+      <c r="D89" s="7" t="s">
+        <v>370</v>
+      </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">

</xml_diff>